<commit_message>
test(formularios): guardar contratos de la calificación final
</commit_message>
<xml_diff>
--- a/src/test/fixtures/forms-responses-http/export.xlsx
+++ b/src/test/fixtures/forms-responses-http/export.xlsx
@@ -39,16 +39,16 @@
     <x:t>date</x:t>
   </x:si>
   <x:si>
-    <x:t>Ta9315f36-000001</x:t>
+    <x:t>Tba6d336f-000001</x:t>
   </x:si>
   <x:si>
     <x:t>Sin información</x:t>
   </x:si>
   <x:si>
-    <x:t>Ta9315f36-000002</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Ta9315f36-000003</x:t>
+    <x:t>Tba6d336f-000002</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Tba6d336f-000003</x:t>
   </x:si>
 </x:sst>
 </file>

</xml_diff>

<commit_message>
test(formularios): actualizar las capturas HTTP del cierre de la etapa 5
</commit_message>
<xml_diff>
--- a/src/test/fixtures/forms-responses-http/export.xlsx
+++ b/src/test/fixtures/forms-responses-http/export.xlsx
@@ -39,16 +39,16 @@
     <x:t>date</x:t>
   </x:si>
   <x:si>
-    <x:t>Tba6d336f-000001</x:t>
+    <x:t>TCC44FCEB-000001</x:t>
   </x:si>
   <x:si>
     <x:t>Sin información</x:t>
   </x:si>
   <x:si>
-    <x:t>Tba6d336f-000002</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Tba6d336f-000003</x:t>
+    <x:t>TCC44FCEB-000002</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TCC44FCEB-000003</x:t>
   </x:si>
 </x:sst>
 </file>

</xml_diff>